<commit_message>
accordions set to open, changed data on sources
</commit_message>
<xml_diff>
--- a/data/sources.xlsx
+++ b/data/sources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aheller\Dropbox\CS\3 - Current Projects\TEA-CART again\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aheller\Documents\GitHub\TEACART\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718C498C-B169-427E-AF54-4FB3661CA61B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC4F8AFF-4B7E-460E-ACA5-069EE1AFE8CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8280C5B7-8E95-43D7-B172-FB4701BB1BAF}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{8280C5B7-8E95-43D7-B172-FB4701BB1BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -498,12 +498,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink 2" xfId="1" xr:uid="{07ED5012-6AD1-42C8-94C1-CB2D4C792F58}"/>
@@ -523,9 +524,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -563,7 +564,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -669,7 +670,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -811,7 +812,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -820,13 +821,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7DB5B7-6594-4B32-9D01-0D9F2F3DF6A4}">
   <dimension ref="A1:C43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="57" customWidth="1"/>
-    <col min="2" max="2" width="127.7109375" customWidth="1"/>
+    <col min="2" max="2" width="127.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -837,7 +838,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="str">
         <f>Sheet2!A2</f>
         <v>American Automobile Association (AAA)</v>
@@ -851,7 +852,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="str">
         <f>Sheet2!A3</f>
         <v>Amtrak</v>
@@ -865,7 +866,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="str">
         <f>Sheet2!A4</f>
         <v>American Public Transportation Association</v>
@@ -879,7 +880,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <f>Sheet2!A5</f>
         <v>Argonne National Laboratory. GREET</v>
@@ -893,7 +894,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <f>Sheet2!A6</f>
         <v>Barr, L.C.</v>
@@ -907,7 +908,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <f>Sheet2!A7</f>
         <v>California Air Pollution Control Officers Association</v>
@@ -921,7 +922,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f>Sheet2!A8</f>
         <v>California Air Resources Board</v>
@@ -935,7 +936,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f>Sheet2!A9</f>
         <v>Cesme, B., R. Roisman, and D. Miller</v>
@@ -949,7 +950,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <f>Sheet2!A10</f>
         <v>Coastal Region MPO</v>
@@ -963,7 +964,7 @@
         <v>2014</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <f>Sheet2!A11</f>
         <v>Cambridge Systematics</v>
@@ -972,12 +973,11 @@
         <f>Sheet2!E11</f>
         <v>&lt;a href="https://www.georgetownclimate.org/files/report/GCC_Investment_Tool.pdf", target=_blank"&gt;Transportation Investment Strategy Tool Documentation, 2021. Prepared for Georgetown Climate Center.&lt;/a&gt;</v>
       </c>
-      <c r="C11" t="str">
-        <f>Sheet2!C11</f>
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C11">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f>Sheet2!A12</f>
         <v>Florida Department of Transportation</v>
@@ -991,7 +991,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f>Sheet2!A13</f>
         <v>Federal Highway Administration</v>
@@ -1005,7 +1005,7 @@
         <v>2013</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f>Sheet2!A14</f>
         <v>Federal Highway Administration</v>
@@ -1019,7 +1019,7 @@
         <v>2014</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="str">
         <f>Sheet2!A15</f>
         <v>McGuckin, N. and A. Fucci</v>
@@ -1033,7 +1033,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f>Sheet2!A16</f>
         <v>Federal Highway Administration</v>
@@ -1047,7 +1047,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
         <f>Sheet2!A17</f>
         <v>FHWA</v>
@@ -1061,7 +1061,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f>Sheet2!A18</f>
         <v>Nicholas, M.</v>
@@ -1075,7 +1075,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f>Sheet2!A19</f>
         <v>Isenstadt, A., et al</v>
@@ -1089,7 +1089,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f>Sheet2!A20</f>
         <v>Mulholland, E.</v>
@@ -1103,7 +1103,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
         <f>Sheet2!A21</f>
         <v>MacArthur, J., C. Cherry, M. Harpool and D. Scheppke.</v>
@@ -1117,7 +1117,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f>Sheet2!A22</f>
         <v>McGuckin, N. and A. Fucci</v>
@@ -1131,7 +1131,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="str">
         <f>Sheet2!A23</f>
         <v>New York City Clean School Bus Coalition</v>
@@ -1145,7 +1145,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="str">
         <f>Sheet2!A24</f>
         <v>NHTS</v>
@@ -1159,7 +1159,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="str">
         <f>Sheet2!A25</f>
         <v>National Highway Traffic Safety Administration</v>
@@ -1173,7 +1173,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="str">
         <f>Sheet2!A26</f>
         <v>Mai, T., et al</v>
@@ -1187,7 +1187,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="str">
         <f>Sheet2!A27</f>
         <v>Johnson, C.; E. Nobler, L. Eudy, and M. Jeffers</v>
@@ -1201,7 +1201,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="str">
         <f>Sheet2!A28</f>
         <v>Hunter, C., et al</v>
@@ -1215,7 +1215,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="str">
         <f>Sheet2!A29</f>
         <v>Federal Transit Administration</v>
@@ -1229,7 +1229,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="str">
         <f>Sheet2!A30</f>
         <v>Oak Ridge National Laboratory</v>
@@ -1243,7 +1243,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="str">
         <f>Sheet2!A31</f>
         <v>Evans, J.E., et al</v>
@@ -1257,7 +1257,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="str">
         <f>Sheet2!A32</f>
         <v>Evans, J.E., and R. H. Pratt, et al</v>
@@ -1271,7 +1271,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="str">
         <f>Sheet2!A33</f>
         <v>[U.K.] Highways Agency</v>
@@ -1285,7 +1285,7 @@
         <v>1997</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="str">
         <f>Sheet2!A34</f>
         <v>U.S. Department of Energy, Energy Information Administration</v>
@@ -1299,7 +1299,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="str">
         <f>Sheet2!A35</f>
         <v>U.S. Department of Energy</v>
@@ -1313,7 +1313,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="str">
         <f>Sheet2!A36</f>
         <v>U.S. Department of Energy</v>
@@ -1327,7 +1327,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="str">
         <f>Sheet2!A37</f>
         <v>U.S. Department of Energy, Alternative Fuels Data Center</v>
@@ -1341,7 +1341,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="str">
         <f>Sheet2!A38</f>
         <v>U.S. Department of Energy, Alternative Fuels Data Center</v>
@@ -1355,7 +1355,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="str">
         <f>Sheet2!A39</f>
         <v>U.S. Department of Transportation</v>
@@ -1369,7 +1369,7 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="str">
         <f>Sheet2!A40</f>
         <v>U.S. Department of Transportation</v>
@@ -1383,7 +1383,7 @@
         <v>2010</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="str">
         <f>Sheet2!A41</f>
         <v>U.S. Environmental Protection Agency</v>
@@ -1397,7 +1397,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="str">
         <f>Sheet2!A42</f>
         <v>Volker, J.N.B., and S.L. Handy</v>
@@ -1411,7 +1411,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="str">
         <f>Sheet2!A43</f>
         <v>Weldon Cooper Center for Public Service, Demographics Research Group</v>
@@ -1434,12 +1434,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A575D46-68C3-4992-B64B-B7045A123F2A}">
   <dimension ref="A1:E43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="39.140625" customWidth="1"/>
+    <col min="1" max="5" width="39.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -1456,7 +1456,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>131</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>&lt;a href="https://gasprices.aaa.com/", target=_blank"&gt;National Average Gas Prices.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>67</v>
       </c>
@@ -1492,7 +1492,7 @@
         <v>&lt;a href="0", target=_blank"&gt;FY2019 Monthly Performance Report.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>&lt;a href="https://www.apta.com/research-technical-resources/transit-statistics/vehicle-database/", target=_blank"&gt;Public Transportation Vehicle Database 2019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>&lt;a href="https://greet.es.anl.gov/", target=_blank"&gt;GREET (Greenhouse gases, Regulated Emissions, and Energy use in Technologies Model). Accessed 2021.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>&lt;a href="https://journals.sagepub.com/doi/10.3141/1706-01", target=_blank"&gt;Testing for the significance of induced highway travel demand in metropolitan areas. Transportation Research Record: Journal of the Transportation Research Board, vol. 1706.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>&lt;a href="https://www.airquality.org/ClimateChange/Documents/Handbook%20Public%20Draft_2021-Aug.pdf", target=_blank"&gt;Handbook for Analyzing Greenhouse Gas Emission Reductions, Assessing Climate Vulnerabilities, and Advancing Health and Equity.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>77</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>&lt;a href="https://ww2.arb.ca.gov/sites/default/files/classic/fuels/lcfs/guidance/lcfsguidance_20-04.pdf", target=_blank"&gt;Low Carbon Fuel Standard (LCFS) Guidance 20-04 Requesting EER-Adjusted Carbon Intensity Using a Tier 2 Pathway Application.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>79</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>&lt;a href="https://journals.sagepub.com/doi/10.1177/0361198118791914", target=_blank"&gt;Strategies and Barriers in Effective Bus Lane Implementation and Management: Best Practices for Use in the Greater Washington, D.C. Region. Transportation Research Record 2672:8.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>81</v>
       </c>
@@ -1618,15 +1618,15 @@
         <v>&lt;a href="https://www.thempc.org/docs/lit/corempo/studies/parkride/2014/aug/tm5.pdf", target=_blank"&gt;Park and Ride Lot Study - Technical Memorandum #5: Financial Analysis and Management Options. Prepared by Connetics Transportation Group, Moffatt &amp; Nichol, and Symbioscity.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>83</v>
       </c>
       <c r="B11" t="s">
         <v>84</v>
       </c>
-      <c r="C11" t="s">
-        <v>42</v>
+      <c r="C11" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="D11" t="s">
         <v>8</v>
@@ -1636,7 +1636,7 @@
         <v>&lt;a href="https://www.georgetownclimate.org/files/report/GCC_Investment_Tool.pdf", target=_blank"&gt;Transportation Investment Strategy Tool Documentation, 2021. Prepared for Georgetown Climate Center.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -1654,7 +1654,7 @@
         <v>&lt;a href="https://www.fdot.gov/programmanagement/estimates/documents/costpermilemodelsreports", target=_blank"&gt;Cost Per Mile Models Reports. Accessed June 2023.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>87</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>&lt;a href="http://www.pedbikesafe.org/PEDSAFE/index.cfm", target=_blank"&gt;PEDSAFE: Pedestrian Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>87</v>
       </c>
@@ -1690,7 +1690,7 @@
         <v>&lt;a href="http://www.pedbikesafe.org/BIKESAFE/index.cfm", target=_blank"&gt;BIKESAFE: Bicycle Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>90</v>
       </c>
@@ -1708,7 +1708,7 @@
         <v>&lt;a href="https://nhts.ornl.gov/assets/2017_nhts_summary_travel_trends.pdf", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>&lt;a href="https://www.fhwa.dot.gov/policyinformation/statistics.cfm", target=_blank"&gt;Highway Statistics Series, 2019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>60</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>&lt;a href="https://faf.ornl.gov/faf5/", target=_blank"&gt;Freight Analysis Framework Version 5.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -1762,7 +1762,7 @@
         <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1780,7 +1780,7 @@
         <v>&lt;a href="https://theicct.org/publication/real-world-phev-us-dec22/", target=_blank"&gt;Real World Usage of Plug-In Hybrid Electric Vehicles. International Council on Clean Transportation.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>98</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>100</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>&lt;a href="https://pdxscholar.library.pdx.edu/trec_reports/161/", target=_blank"&gt;A North American Survey of Electric Bicycle Owners. NITC-RR-1041. Portland, OR: Transportation Research and Education Center (TREC). https://dx.doi.org/10.15760/ trec.197&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>90</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>&lt;a href="0", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>56</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>57</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>103</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>&lt;a href="https://www.nrel.gov/docs/fy18osti/71500.pdf", target=_blank"&gt;Electrification Futures Study: Scenarios of Electric Technology Adoption and Power Consumption for the United States. Golden, CO: National Renewable Energy Laboratory. NREL/TP-6A20-71500.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>105</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>&lt;a href="https://afdc.energy.gov/files/u/publication/financial_analysis_be_transit_buses.pdf", target=_blank"&gt;Financial Analysis of Battery Electric Transit Buses. National Renewable Energy Laboratory Technical Report NREL/TP-5400-74832.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>107</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>&lt;a href="https://www.nrel.gov/docs/fy21osti/71796.pdf", target=_blank"&gt;Spatial and Temporal Analysis of the Total Cost of Ownership for Class 8 Tractors and Class 4 Parcel Delivery Trucks. National Renewable Energy Laboratory Technical Report NREL/TP-5400-71796.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>133</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>&lt;a href="https://www.transit.dot.gov/ntd", target=_blank"&gt;National Transit Database&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>109</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>&lt;a href="https://tedb.ornl.gov/data/", target=_blank"&gt;Transportation Energy Data Book, Edition 40.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>111</v>
       </c>
@@ -1996,7 +1996,7 @@
         <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 9: Transit Scheduling and Frequency. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>113</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 5: Vanpools and Buspools. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>115</v>
       </c>
@@ -2032,7 +2032,7 @@
         <v>&lt;a href="0", target=_blank"&gt;Design Manual for Roads and Bridges, Volume 12, Section 2, Part 2: Induced Traffic Appraisal.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>117</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>61</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>61</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>62</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>62</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>121</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>&lt;a href="https://www.itskrs.its.dot.gov/its/benecost.nsf/ID/5551ecb16b1bc9698525725f007a75d0", target=_blank"&gt;The cost of retiming traffic signals in the Washington, DC area is about $3,500 per intersection. ITS Deployment Evaluation, Intelligent Transportation Systems Joint Program Office.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>121</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>&lt;a href="http://www.reconnectingamerica.org/assets/Uploads/DOTClimateChangeReport-April2010-Volume1and2.pdf", target=_blank"&gt;Transportation's Role in Reducing U.S. Greenhouse Gas Emissions.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>124</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>&lt;a href="https://www.epa.gov/climateleadership/ghg-emission-factors-hub", target=_blank"&gt;GHG Emission Factors Hub.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>126</v>
       </c>
@@ -2194,7 +2194,7 @@
         <v>&lt;a href="https://escholarship.org/uc/item/1hh9b9mf", target=_blank"&gt;Updating the Induced Travel Calculator. National Center for Sustainable Transportation and UC Davis.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
updates to sources and expanded names for funding table
</commit_message>
<xml_diff>
--- a/data/sources.xlsx
+++ b/data/sources.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aheller\Documents\GitHub\TEACART\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC4F8AFF-4B7E-460E-ACA5-069EE1AFE8CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5305AE1-94FD-42C4-BC45-86AEDBD4C8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{8280C5B7-8E95-43D7-B172-FB4701BB1BAF}"/>
   </bookViews>
@@ -294,9 +294,6 @@
     <t>Cambridge Systematics</t>
   </si>
   <si>
-    <t>Transportation Investment Strategy Tool Documentation, 2021. Prepared for Georgetown Climate Center.</t>
-  </si>
-  <si>
     <t>Florida Department of Transportation</t>
   </si>
   <si>
@@ -442,6 +439,9 @@
   </si>
   <si>
     <t>Federal Transit Administration</t>
+  </si>
+  <si>
+    <t>Transportation Investment Strategy Tool Documentation, 2023. Prepared for Georgetown Climate Center.</t>
   </si>
 </sst>
 </file>
@@ -821,13 +821,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7DB5B7-6594-4B32-9D01-0D9F2F3DF6A4}">
   <dimension ref="A1:C43"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="57" customWidth="1"/>
-    <col min="2" max="2" width="127.6640625" customWidth="1"/>
+    <col min="2" max="2" width="127.6796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -838,35 +838,35 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A2" t="str">
         <f>Sheet2!A2</f>
-        <v>American Automobile Association (AAA)</v>
+        <v>[U.K.] Highways Agency</v>
       </c>
       <c r="B2" t="str">
         <f>Sheet2!E2</f>
-        <v>&lt;a href="https://gasprices.aaa.com/", target=_blank"&gt;National Average Gas Prices.&lt;/a&gt;</v>
+        <v>&lt;a href="0", target=_blank"&gt;Design Manual for Roads and Bridges, Volume 12, Section 2, Part 2: Induced Traffic Appraisal.&lt;/a&gt;</v>
       </c>
       <c r="C2" t="str">
         <f>Sheet2!C2</f>
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A3" t="str">
         <f>Sheet2!A3</f>
-        <v>Amtrak</v>
+        <v>American Automobile Association (AAA)</v>
       </c>
       <c r="B3" t="str">
         <f>Sheet2!E3</f>
-        <v>&lt;a href="0", target=_blank"&gt;FY2019 Monthly Performance Report.&lt;/a&gt;</v>
+        <v>&lt;a href="https://gasprices.aaa.com/", target=_blank"&gt;National Average Gas Prices.&lt;/a&gt;</v>
       </c>
       <c r="C3" t="str">
         <f>Sheet2!C3</f>
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A4" t="str">
         <f>Sheet2!A4</f>
         <v>American Public Transportation Association</v>
@@ -880,160 +880,161 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A5" t="str">
         <f>Sheet2!A5</f>
-        <v>Argonne National Laboratory. GREET</v>
+        <v>Amtrak</v>
       </c>
       <c r="B5" t="str">
         <f>Sheet2!E5</f>
-        <v>&lt;a href="https://greet.es.anl.gov/", target=_blank"&gt;GREET (Greenhouse gases, Regulated Emissions, and Energy use in Technologies Model). Accessed 2021.&lt;/a&gt;</v>
+        <v>&lt;a href="0", target=_blank"&gt;FY2019 Monthly Performance Report.&lt;/a&gt;</v>
       </c>
       <c r="C5" t="str">
         <f>Sheet2!C5</f>
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A6" t="str">
         <f>Sheet2!A6</f>
-        <v>Barr, L.C.</v>
+        <v>Argonne National Laboratory. GREET</v>
       </c>
       <c r="B6" t="str">
         <f>Sheet2!E6</f>
-        <v>&lt;a href="https://journals.sagepub.com/doi/10.3141/1706-01", target=_blank"&gt;Testing for the significance of induced highway travel demand in metropolitan areas. Transportation Research Record: Journal of the Transportation Research Board, vol. 1706.&lt;/a&gt;</v>
+        <v>&lt;a href="https://greet.es.anl.gov/", target=_blank"&gt;GREET (Greenhouse gases, Regulated Emissions, and Energy use in Technologies Model). Accessed 2021.&lt;/a&gt;</v>
       </c>
       <c r="C6" t="str">
         <f>Sheet2!C6</f>
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A7" t="str">
         <f>Sheet2!A7</f>
-        <v>California Air Pollution Control Officers Association</v>
+        <v>Barr, L.C.</v>
       </c>
       <c r="B7" t="str">
         <f>Sheet2!E7</f>
-        <v>&lt;a href="https://www.airquality.org/ClimateChange/Documents/Handbook%20Public%20Draft_2021-Aug.pdf", target=_blank"&gt;Handbook for Analyzing Greenhouse Gas Emission Reductions, Assessing Climate Vulnerabilities, and Advancing Health and Equity.&lt;/a&gt;</v>
+        <v>&lt;a href="https://journals.sagepub.com/doi/10.3141/1706-01", target=_blank"&gt;Testing for the significance of induced highway travel demand in metropolitan areas. Transportation Research Record: Journal of the Transportation Research Board, vol. 1706.&lt;/a&gt;</v>
       </c>
       <c r="C7" t="str">
         <f>Sheet2!C7</f>
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A8" t="str">
         <f>Sheet2!A8</f>
-        <v>California Air Resources Board</v>
+        <v>California Air Pollution Control Officers Association</v>
       </c>
       <c r="B8" t="str">
         <f>Sheet2!E8</f>
-        <v>&lt;a href="https://ww2.arb.ca.gov/sites/default/files/classic/fuels/lcfs/guidance/lcfsguidance_20-04.pdf", target=_blank"&gt;Low Carbon Fuel Standard (LCFS) Guidance 20-04 Requesting EER-Adjusted Carbon Intensity Using a Tier 2 Pathway Application.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.airquality.org/ClimateChange/Documents/Handbook%20Public%20Draft_2021-Aug.pdf", target=_blank"&gt;Handbook for Analyzing Greenhouse Gas Emission Reductions, Assessing Climate Vulnerabilities, and Advancing Health and Equity.&lt;/a&gt;</v>
       </c>
       <c r="C8" t="str">
         <f>Sheet2!C8</f>
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A9" t="str">
         <f>Sheet2!A9</f>
-        <v>Cesme, B., R. Roisman, and D. Miller</v>
+        <v>California Air Resources Board</v>
       </c>
       <c r="B9" t="str">
         <f>Sheet2!E9</f>
-        <v>&lt;a href="https://journals.sagepub.com/doi/10.1177/0361198118791914", target=_blank"&gt;Strategies and Barriers in Effective Bus Lane Implementation and Management: Best Practices for Use in the Greater Washington, D.C. Region. Transportation Research Record 2672:8.&lt;/a&gt;</v>
+        <v>&lt;a href="https://ww2.arb.ca.gov/sites/default/files/classic/fuels/lcfs/guidance/lcfsguidance_20-04.pdf", target=_blank"&gt;Low Carbon Fuel Standard (LCFS) Guidance 20-04 Requesting EER-Adjusted Carbon Intensity Using a Tier 2 Pathway Application.&lt;/a&gt;</v>
       </c>
       <c r="C9" t="str">
         <f>Sheet2!C9</f>
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A10" t="str">
         <f>Sheet2!A10</f>
-        <v>Coastal Region MPO</v>
+        <v>Cambridge Systematics</v>
       </c>
       <c r="B10" t="str">
         <f>Sheet2!E10</f>
-        <v>&lt;a href="https://www.thempc.org/docs/lit/corempo/studies/parkride/2014/aug/tm5.pdf", target=_blank"&gt;Park and Ride Lot Study - Technical Memorandum #5: Financial Analysis and Management Options. Prepared by Connetics Transportation Group, Moffatt &amp; Nichol, and Symbioscity.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.georgetownclimate.org/files/report/GCC_Investment_Tool.pdf", target=_blank"&gt;Transportation Investment Strategy Tool Documentation, 2023. Prepared for Georgetown Climate Center.&lt;/a&gt;</v>
       </c>
       <c r="C10" t="str">
         <f>Sheet2!C10</f>
-        <v>2014</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A11" t="str">
         <f>Sheet2!A11</f>
-        <v>Cambridge Systematics</v>
+        <v>Cesme, B., R. Roisman, and D. Miller</v>
       </c>
       <c r="B11" t="str">
         <f>Sheet2!E11</f>
-        <v>&lt;a href="https://www.georgetownclimate.org/files/report/GCC_Investment_Tool.pdf", target=_blank"&gt;Transportation Investment Strategy Tool Documentation, 2021. Prepared for Georgetown Climate Center.&lt;/a&gt;</v>
-      </c>
-      <c r="C11">
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://journals.sagepub.com/doi/10.1177/0361198118791914", target=_blank"&gt;Strategies and Barriers in Effective Bus Lane Implementation and Management: Best Practices for Use in the Greater Washington, D.C. Region. Transportation Research Record 2672:8.&lt;/a&gt;</v>
+      </c>
+      <c r="C11" t="str">
+        <f>Sheet2!C11</f>
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A12" t="str">
         <f>Sheet2!A12</f>
-        <v>Florida Department of Transportation</v>
+        <v>Coastal Region MPO</v>
       </c>
       <c r="B12" t="str">
         <f>Sheet2!E12</f>
-        <v>&lt;a href="https://www.fdot.gov/programmanagement/estimates/documents/costpermilemodelsreports", target=_blank"&gt;Cost Per Mile Models Reports. Accessed June 2023.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.thempc.org/docs/lit/corempo/studies/parkride/2014/aug/tm5.pdf", target=_blank"&gt;Park and Ride Lot Study - Technical Memorandum #5: Financial Analysis and Management Options. Prepared by Connetics Transportation Group, Moffatt &amp; Nichol, and Symbioscity.&lt;/a&gt;</v>
       </c>
       <c r="C12" t="str">
         <f>Sheet2!C12</f>
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A13" t="str">
         <f>Sheet2!A13</f>
-        <v>Federal Highway Administration</v>
+        <v>Evans, J.E., and R. H. Pratt, et al</v>
       </c>
       <c r="B13" t="str">
         <f>Sheet2!E13</f>
-        <v>&lt;a href="http://www.pedbikesafe.org/PEDSAFE/index.cfm", target=_blank"&gt;PEDSAFE: Pedestrian Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 5: Vanpools and Buspools. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
       </c>
       <c r="C13" t="str">
         <f>Sheet2!C13</f>
-        <v>2013</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A14" t="str">
         <f>Sheet2!A14</f>
-        <v>Federal Highway Administration</v>
+        <v>Evans, J.E., et al</v>
       </c>
       <c r="B14" t="str">
         <f>Sheet2!E14</f>
-        <v>&lt;a href="http://www.pedbikesafe.org/BIKESAFE/index.cfm", target=_blank"&gt;BIKESAFE: Bicycle Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 9: Transit Scheduling and Frequency. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
       </c>
       <c r="C14" t="str">
         <f>Sheet2!C14</f>
-        <v>2014</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A15" t="str">
         <f>Sheet2!A15</f>
-        <v>McGuckin, N. and A. Fucci</v>
+        <v>Federal Highway Administration</v>
       </c>
       <c r="B15" t="str">
         <f>Sheet2!E15</f>
-        <v>&lt;a href="https://nhts.ornl.gov/assets/2017_nhts_summary_travel_trends.pdf", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
+        <v>&lt;a href="http://www.pedbikesafe.org/BIKESAFE/index.cfm", target=_blank"&gt;BIKESAFE: Bicycle Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
       </c>
       <c r="C15" t="str">
         <f>Sheet2!C15</f>
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A16" t="str">
         <f>Sheet2!A16</f>
         <v>Federal Highway Administration</v>
@@ -1047,315 +1048,315 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A17" t="str">
         <f>Sheet2!A17</f>
-        <v>FHWA</v>
+        <v>Federal Highway Administration</v>
       </c>
       <c r="B17" t="str">
         <f>Sheet2!E17</f>
-        <v>&lt;a href="https://faf.ornl.gov/faf5/", target=_blank"&gt;Freight Analysis Framework Version 5.&lt;/a&gt;</v>
+        <v>&lt;a href="http://www.pedbikesafe.org/PEDSAFE/index.cfm", target=_blank"&gt;PEDSAFE: Pedestrian Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
       </c>
       <c r="C17" t="str">
         <f>Sheet2!C17</f>
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A18" t="str">
         <f>Sheet2!A18</f>
-        <v>Nicholas, M.</v>
+        <v>Federal Transit Administration</v>
       </c>
       <c r="B18" t="str">
         <f>Sheet2!E18</f>
-        <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.transit.dot.gov/ntd", target=_blank"&gt;National Transit Database&lt;/a&gt;</v>
       </c>
       <c r="C18" t="str">
         <f>Sheet2!C18</f>
         <v>2019</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A19" t="str">
         <f>Sheet2!A19</f>
-        <v>Isenstadt, A., et al</v>
+        <v>FHWA</v>
       </c>
       <c r="B19" t="str">
         <f>Sheet2!E19</f>
-        <v>&lt;a href="https://theicct.org/publication/real-world-phev-us-dec22/", target=_blank"&gt;Real World Usage of Plug-In Hybrid Electric Vehicles. International Council on Clean Transportation.&lt;/a&gt;</v>
+        <v>&lt;a href="https://faf.ornl.gov/faf5/", target=_blank"&gt;Freight Analysis Framework Version 5.&lt;/a&gt;</v>
       </c>
       <c r="C19" t="str">
         <f>Sheet2!C19</f>
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A20" t="str">
         <f>Sheet2!A20</f>
-        <v>Mulholland, E.</v>
+        <v>Florida Department of Transportation</v>
       </c>
       <c r="B20" t="str">
         <f>Sheet2!E20</f>
-        <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.fdot.gov/programmanagement/estimates/documents/costpermilemodelsreports", target=_blank"&gt;Cost Per Mile Models Reports. Accessed June 2023.&lt;/a&gt;</v>
       </c>
       <c r="C20" t="str">
         <f>Sheet2!C20</f>
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A21" t="str">
         <f>Sheet2!A21</f>
-        <v>MacArthur, J., C. Cherry, M. Harpool and D. Scheppke.</v>
+        <v>Hunter, C., et al</v>
       </c>
       <c r="B21" t="str">
         <f>Sheet2!E21</f>
-        <v>&lt;a href="https://pdxscholar.library.pdx.edu/trec_reports/161/", target=_blank"&gt;A North American Survey of Electric Bicycle Owners. NITC-RR-1041. Portland, OR: Transportation Research and Education Center (TREC). https://dx.doi.org/10.15760/ trec.197&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.nrel.gov/docs/fy21osti/71796.pdf", target=_blank"&gt;Spatial and Temporal Analysis of the Total Cost of Ownership for Class 8 Tractors and Class 4 Parcel Delivery Trucks. National Renewable Energy Laboratory Technical Report NREL/TP-5400-71796.&lt;/a&gt;</v>
       </c>
       <c r="C21" t="str">
         <f>Sheet2!C21</f>
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A22" t="str">
         <f>Sheet2!A22</f>
-        <v>McGuckin, N. and A. Fucci</v>
+        <v>Isenstadt, A., et al</v>
       </c>
       <c r="B22" t="str">
         <f>Sheet2!E22</f>
-        <v>&lt;a href="0", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
+        <v>&lt;a href="https://theicct.org/publication/real-world-phev-us-dec22/", target=_blank"&gt;Real World Usage of Plug-In Hybrid Electric Vehicles. International Council on Clean Transportation.&lt;/a&gt;</v>
       </c>
       <c r="C22" t="str">
         <f>Sheet2!C22</f>
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A23" t="str">
         <f>Sheet2!A23</f>
-        <v>New York City Clean School Bus Coalition</v>
+        <v>Johnson, C.; E. Nobler, L. Eudy, and M. Jeffers</v>
       </c>
       <c r="B23" t="str">
         <f>Sheet2!E23</f>
-        <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
+        <v>&lt;a href="https://afdc.energy.gov/files/u/publication/financial_analysis_be_transit_buses.pdf", target=_blank"&gt;Financial Analysis of Battery Electric Transit Buses. National Renewable Energy Laboratory Technical Report NREL/TP-5400-74832.&lt;/a&gt;</v>
       </c>
       <c r="C23" t="str">
         <f>Sheet2!C23</f>
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A24" t="str">
         <f>Sheet2!A24</f>
-        <v>NHTS</v>
+        <v>MacArthur, J., C. Cherry, M. Harpool and D. Scheppke.</v>
       </c>
       <c r="B24" t="str">
         <f>Sheet2!E24</f>
-        <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
+        <v>&lt;a href="https://pdxscholar.library.pdx.edu/trec_reports/161/", target=_blank"&gt;A North American Survey of Electric Bicycle Owners. NITC-RR-1041. Portland, OR: Transportation Research and Education Center (TREC). https://dx.doi.org/10.15760/ trec.197&lt;/a&gt;</v>
       </c>
       <c r="C24" t="str">
         <f>Sheet2!C24</f>
-        <v>2009</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A25" t="str">
         <f>Sheet2!A25</f>
-        <v>National Highway Traffic Safety Administration</v>
+        <v>Mai, T., et al</v>
       </c>
       <c r="B25" t="str">
         <f>Sheet2!E25</f>
-        <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.nrel.gov/docs/fy18osti/71500.pdf", target=_blank"&gt;Electrification Futures Study: Scenarios of Electric Technology Adoption and Power Consumption for the United States. Golden, CO: National Renewable Energy Laboratory. NREL/TP-6A20-71500.&lt;/a&gt;</v>
       </c>
       <c r="C25" t="str">
         <f>Sheet2!C25</f>
-        <v>2015</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A26" t="str">
         <f>Sheet2!A26</f>
-        <v>Mai, T., et al</v>
+        <v>McGuckin, N. and A. Fucci</v>
       </c>
       <c r="B26" t="str">
         <f>Sheet2!E26</f>
-        <v>&lt;a href="https://www.nrel.gov/docs/fy18osti/71500.pdf", target=_blank"&gt;Electrification Futures Study: Scenarios of Electric Technology Adoption and Power Consumption for the United States. Golden, CO: National Renewable Energy Laboratory. NREL/TP-6A20-71500.&lt;/a&gt;</v>
+        <v>&lt;a href="https://nhts.ornl.gov/assets/2017_nhts_summary_travel_trends.pdf", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
       </c>
       <c r="C26" t="str">
         <f>Sheet2!C26</f>
         <v>2018</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A27" t="str">
         <f>Sheet2!A27</f>
-        <v>Johnson, C.; E. Nobler, L. Eudy, and M. Jeffers</v>
+        <v>McGuckin, N. and A. Fucci</v>
       </c>
       <c r="B27" t="str">
         <f>Sheet2!E27</f>
-        <v>&lt;a href="https://afdc.energy.gov/files/u/publication/financial_analysis_be_transit_buses.pdf", target=_blank"&gt;Financial Analysis of Battery Electric Transit Buses. National Renewable Energy Laboratory Technical Report NREL/TP-5400-74832.&lt;/a&gt;</v>
+        <v>&lt;a href="0", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
       </c>
       <c r="C27" t="str">
         <f>Sheet2!C27</f>
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A28" t="str">
         <f>Sheet2!A28</f>
-        <v>Hunter, C., et al</v>
+        <v>Mulholland, E.</v>
       </c>
       <c r="B28" t="str">
         <f>Sheet2!E28</f>
-        <v>&lt;a href="https://www.nrel.gov/docs/fy21osti/71796.pdf", target=_blank"&gt;Spatial and Temporal Analysis of the Total Cost of Ownership for Class 8 Tractors and Class 4 Parcel Delivery Trucks. National Renewable Energy Laboratory Technical Report NREL/TP-5400-71796.&lt;/a&gt;</v>
+        <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
       </c>
       <c r="C28" t="str">
         <f>Sheet2!C28</f>
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A29" t="str">
         <f>Sheet2!A29</f>
-        <v>Federal Transit Administration</v>
+        <v>National Highway Traffic Safety Administration</v>
       </c>
       <c r="B29" t="str">
         <f>Sheet2!E29</f>
-        <v>&lt;a href="https://www.transit.dot.gov/ntd", target=_blank"&gt;National Transit Database&lt;/a&gt;</v>
+        <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
       </c>
       <c r="C29" t="str">
         <f>Sheet2!C29</f>
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A30" t="str">
         <f>Sheet2!A30</f>
-        <v>Oak Ridge National Laboratory</v>
+        <v>New York City Clean School Bus Coalition</v>
       </c>
       <c r="B30" t="str">
         <f>Sheet2!E30</f>
-        <v>&lt;a href="https://tedb.ornl.gov/data/", target=_blank"&gt;Transportation Energy Data Book, Edition 40.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
       </c>
       <c r="C30" t="str">
         <f>Sheet2!C30</f>
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A31" t="str">
         <f>Sheet2!A31</f>
-        <v>Evans, J.E., et al</v>
+        <v>NHTS</v>
       </c>
       <c r="B31" t="str">
         <f>Sheet2!E31</f>
-        <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 9: Transit Scheduling and Frequency. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
+        <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
       </c>
       <c r="C31" t="str">
         <f>Sheet2!C31</f>
-        <v>2004</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2009</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A32" t="str">
         <f>Sheet2!A32</f>
-        <v>Evans, J.E., and R. H. Pratt, et al</v>
+        <v>Nicholas, M.</v>
       </c>
       <c r="B32" t="str">
         <f>Sheet2!E32</f>
-        <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 5: Vanpools and Buspools. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
+        <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
       </c>
       <c r="C32" t="str">
         <f>Sheet2!C32</f>
-        <v>2005</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A33" t="str">
         <f>Sheet2!A33</f>
-        <v>[U.K.] Highways Agency</v>
+        <v>Oak Ridge National Laboratory</v>
       </c>
       <c r="B33" t="str">
         <f>Sheet2!E33</f>
-        <v>&lt;a href="0", target=_blank"&gt;Design Manual for Roads and Bridges, Volume 12, Section 2, Part 2: Induced Traffic Appraisal.&lt;/a&gt;</v>
+        <v>&lt;a href="https://tedb.ornl.gov/data/", target=_blank"&gt;Transportation Energy Data Book, Edition 40.&lt;/a&gt;</v>
       </c>
       <c r="C33" t="str">
         <f>Sheet2!C33</f>
-        <v>1997</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A34" t="str">
         <f>Sheet2!A34</f>
-        <v>U.S. Department of Energy, Energy Information Administration</v>
+        <v>U.S. Department of Energy</v>
       </c>
       <c r="B34" t="str">
         <f>Sheet2!E34</f>
-        <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
       </c>
       <c r="C34" t="str">
         <f>Sheet2!C34</f>
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A35" t="str">
         <f>Sheet2!A35</f>
         <v>U.S. Department of Energy</v>
       </c>
       <c r="B35" t="str">
         <f>Sheet2!E35</f>
-        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
       </c>
       <c r="C35" t="str">
         <f>Sheet2!C35</f>
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A36" t="str">
         <f>Sheet2!A36</f>
-        <v>U.S. Department of Energy</v>
+        <v>U.S. Department of Energy, Alternative Fuels Data Center</v>
       </c>
       <c r="B36" t="str">
         <f>Sheet2!E36</f>
-        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
+        <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
       </c>
       <c r="C36" t="str">
         <f>Sheet2!C36</f>
         <v>2023</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A37" t="str">
         <f>Sheet2!A37</f>
         <v>U.S. Department of Energy, Alternative Fuels Data Center</v>
       </c>
       <c r="B37" t="str">
         <f>Sheet2!E37</f>
-        <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
+        <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
       </c>
       <c r="C37" t="str">
         <f>Sheet2!C37</f>
         <v>2023</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A38" t="str">
         <f>Sheet2!A38</f>
-        <v>U.S. Department of Energy, Alternative Fuels Data Center</v>
+        <v>U.S. Department of Energy, Energy Information Administration</v>
       </c>
       <c r="B38" t="str">
         <f>Sheet2!E38</f>
-        <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
       </c>
       <c r="C38" t="str">
         <f>Sheet2!C38</f>
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A39" t="str">
         <f>Sheet2!A39</f>
         <v>U.S. Department of Transportation</v>
@@ -1369,7 +1370,7 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A40" t="str">
         <f>Sheet2!A40</f>
         <v>U.S. Department of Transportation</v>
@@ -1383,7 +1384,7 @@
         <v>2010</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A41" t="str">
         <f>Sheet2!A41</f>
         <v>U.S. Environmental Protection Agency</v>
@@ -1397,7 +1398,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A42" t="str">
         <f>Sheet2!A42</f>
         <v>Volker, J.N.B., and S.L. Handy</v>
@@ -1411,7 +1412,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A43" t="str">
         <f>Sheet2!A43</f>
         <v>Weldon Cooper Center for Public Service, Demographics Research Group</v>
@@ -1434,12 +1435,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A575D46-68C3-4992-B64B-B7045A123F2A}">
   <dimension ref="A1:E43"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="5" width="39.109375" customWidth="1"/>
+    <col min="1" max="5" width="39.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -1453,46 +1454,46 @@
         <v>39</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>115</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="str">
         <f>_xlfn.CONCAT("&lt;a href=",CHAR(34),D2,CHAR(34),", target=_blank",CHAR(34),"&gt;",B2,"&lt;/a&gt;")</f>
-        <v>&lt;a href="https://gasprices.aaa.com/", target=_blank"&gt;National Average Gas Prices.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="0", target=_blank"&gt;Design Manual for Roads and Bridges, Volume 12, Section 2, Part 2: Induced Traffic Appraisal.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>130</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3">
+        <v>40</v>
+      </c>
+      <c r="D3" t="s">
         <v>0</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" ref="E3:E43" si="0">_xlfn.CONCAT("&lt;a href=",CHAR(34),D3,CHAR(34),", target=_blank",CHAR(34),"&gt;",B3,"&lt;/a&gt;")</f>
-        <v>&lt;a href="0", target=_blank"&gt;FY2019 Monthly Performance Report.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://gasprices.aaa.com/", target=_blank"&gt;National Average Gas Prices.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -1510,210 +1511,210 @@
         <v>&lt;a href="https://www.apta.com/research-technical-resources/transit-statistics/vehicle-database/", target=_blank"&gt;Public Transportation Vehicle Database 2019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="0", target=_blank"&gt;FY2019 Monthly Performance Report.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
         <v>71</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>72</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>42</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>2</v>
       </c>
-      <c r="E5" t="str">
+      <c r="E6" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://greet.es.anl.gov/", target=_blank"&gt;GREET (Greenhouse gases, Regulated Emissions, and Energy use in Technologies Model). Accessed 2021.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
         <v>73</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>74</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>43</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D7" t="s">
         <v>3</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E7" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://journals.sagepub.com/doi/10.3141/1706-01", target=_blank"&gt;Testing for the significance of induced highway travel demand in metropolitan areas. Transportation Research Record: Journal of the Transportation Research Board, vol. 1706.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A8" t="s">
         <v>75</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>76</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>42</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>4</v>
       </c>
-      <c r="E7" t="str">
+      <c r="E8" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://www.airquality.org/ClimateChange/Documents/Handbook%20Public%20Draft_2021-Aug.pdf", target=_blank"&gt;Handbook for Analyzing Greenhouse Gas Emission Reductions, Assessing Climate Vulnerabilities, and Advancing Health and Equity.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A9" t="s">
         <v>77</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>78</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>44</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D9" t="s">
         <v>5</v>
       </c>
-      <c r="E8" t="str">
+      <c r="E9" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://ww2.arb.ca.gov/sites/default/files/classic/fuels/lcfs/guidance/lcfsguidance_20-04.pdf", target=_blank"&gt;Low Carbon Fuel Standard (LCFS) Guidance 20-04 Requesting EER-Adjusted Carbon Intensity Using a Tier 2 Pathway Application.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://www.georgetownclimate.org/files/report/GCC_Investment_Tool.pdf", target=_blank"&gt;Transportation Investment Strategy Tool Documentation, 2023. Prepared for Georgetown Climate Center.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A11" t="s">
         <v>79</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B11" t="s">
         <v>80</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C11" t="s">
         <v>45</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D11" t="s">
         <v>6</v>
       </c>
-      <c r="E9" t="str">
+      <c r="E11" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://journals.sagepub.com/doi/10.1177/0361198118791914", target=_blank"&gt;Strategies and Barriers in Effective Bus Lane Implementation and Management: Best Practices for Use in the Greater Washington, D.C. Region. Transportation Research Record 2672:8.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A12" t="s">
         <v>81</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B12" t="s">
         <v>82</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C12" t="s">
         <v>46</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D12" t="s">
         <v>7</v>
       </c>
-      <c r="E10" t="str">
+      <c r="E12" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://www.thempc.org/docs/lit/corempo/studies/parkride/2014/aug/tm5.pdf", target=_blank"&gt;Park and Ride Lot Study - Technical Memorandum #5: Financial Analysis and Management Options. Prepared by Connetics Transportation Group, Moffatt &amp; Nichol, and Symbioscity.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B11" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.georgetownclimate.org/files/report/GCC_Investment_Tool.pdf", target=_blank"&gt;Transportation Investment Strategy Tool Documentation, 2021. Prepared for Georgetown Climate Center.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 5: Vanpools and Buspools. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 9: Transit Scheduling and Frequency. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A15" t="s">
         <v>86</v>
       </c>
-      <c r="C12" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.fdot.gov/programmanagement/estimates/documents/costpermilemodelsreports", target=_blank"&gt;Cost Per Mile Models Reports. Accessed June 2023.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>87</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="B15" t="s">
         <v>88</v>
       </c>
-      <c r="C13" t="s">
-        <v>48</v>
-      </c>
-      <c r="D13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="http://www.pedbikesafe.org/PEDSAFE/index.cfm", target=_blank"&gt;PEDSAFE: Pedestrian Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" t="s">
-        <v>89</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>46</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D15" t="s">
         <v>11</v>
       </c>
-      <c r="E14" t="str">
+      <c r="E15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="http://www.pedbikesafe.org/BIKESAFE/index.cfm", target=_blank"&gt;BIKESAFE: Bicycle Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B15" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" t="s">
         <v>91</v>
-      </c>
-      <c r="C15" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://nhts.ornl.gov/assets/2017_nhts_summary_travel_trends.pdf", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>87</v>
-      </c>
-      <c r="B16" t="s">
-        <v>92</v>
       </c>
       <c r="C16" t="s">
         <v>41</v>
@@ -1726,331 +1727,331 @@
         <v>&lt;a href="https://www.fhwa.dot.gov/policyinformation/statistics.cfm", target=_blank"&gt;Highway Statistics Series, 2019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E17" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://faf.ornl.gov/faf5/", target=_blank"&gt;Freight Analysis Framework Version 5.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="http://www.pedbikesafe.org/PEDSAFE/index.cfm", target=_blank"&gt;PEDSAFE: Pedestrian Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>131</v>
       </c>
       <c r="C18" t="s">
         <v>41</v>
       </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://www.transit.dot.gov/ntd", target=_blank"&gt;National Transit Database&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A19" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://faf.ornl.gov/faf5/", target=_blank"&gt;Freight Analysis Framework Version 5.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://www.fdot.gov/programmanagement/estimates/documents/costpermilemodelsreports", target=_blank"&gt;Cost Per Mile Models Reports. Accessed June 2023.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A21" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://www.nrel.gov/docs/fy21osti/71796.pdf", target=_blank"&gt;Spatial and Temporal Analysis of the Total Cost of Ownership for Class 8 Tractors and Class 4 Parcel Delivery Trucks. National Renewable Energy Laboratory Technical Report NREL/TP-5400-71796.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" t="s">
         <v>96</v>
       </c>
-      <c r="B19" t="s">
-        <v>97</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="C22" t="s">
         <v>40</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D22" t="s">
         <v>16</v>
       </c>
-      <c r="E19" t="str">
+      <c r="E22" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://theicct.org/publication/real-world-phev-us-dec22/", target=_blank"&gt;Real World Usage of Plug-In Hybrid Electric Vehicles. International Council on Clean Transportation.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>98</v>
-      </c>
-      <c r="B20" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A23" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" t="s">
+        <v>105</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://afdc.energy.gov/files/u/publication/financial_analysis_be_transit_buses.pdf", target=_blank"&gt;Financial Analysis of Battery Electric Transit Buses. National Renewable Energy Laboratory Technical Report NREL/TP-5400-74832.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A24" t="s">
         <v>99</v>
       </c>
-      <c r="C20" t="s">
-        <v>40</v>
-      </c>
-      <c r="D20" t="s">
-        <v>17</v>
-      </c>
-      <c r="E20" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="B24" t="s">
         <v>100</v>
       </c>
-      <c r="B21" t="s">
-        <v>101</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="C24" t="s">
         <v>45</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D24" t="s">
         <v>18</v>
       </c>
-      <c r="E21" t="str">
+      <c r="E24" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://pdxscholar.library.pdx.edu/trec_reports/161/", target=_blank"&gt;A North American Survey of Electric Bicycle Owners. NITC-RR-1041. Portland, OR: Transportation Research and Education Center (TREC). https://dx.doi.org/10.15760/ trec.197&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A25" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" t="s">
+        <v>103</v>
+      </c>
+      <c r="C25" t="s">
+        <v>45</v>
+      </c>
+      <c r="D25" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://www.nrel.gov/docs/fy18osti/71500.pdf", target=_blank"&gt;Electrification Futures Study: Scenarios of Electric Technology Adoption and Power Consumption for the United States. Golden, CO: National Renewable Energy Laboratory. NREL/TP-6A20-71500.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A26" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" t="s">
         <v>90</v>
-      </c>
-      <c r="B22" t="s">
-        <v>91</v>
-      </c>
-      <c r="C22" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="0", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" t="s">
-        <v>102</v>
-      </c>
-      <c r="C23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" t="s">
-        <v>20</v>
-      </c>
-      <c r="E23" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>56</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" t="s">
-        <v>49</v>
-      </c>
-      <c r="D24">
-        <v>0</v>
-      </c>
-      <c r="E24" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>57</v>
-      </c>
-      <c r="B25" t="s">
-        <v>58</v>
-      </c>
-      <c r="C25" t="s">
-        <v>50</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>103</v>
-      </c>
-      <c r="B26" t="s">
-        <v>104</v>
       </c>
       <c r="C26" t="s">
         <v>45</v>
       </c>
       <c r="D26" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E26" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.nrel.gov/docs/fy18osti/71500.pdf", target=_blank"&gt;Electrification Futures Study: Scenarios of Electric Technology Adoption and Power Consumption for the United States. Golden, CO: National Renewable Energy Laboratory. NREL/TP-6A20-71500.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://nhts.ornl.gov/assets/2017_nhts_summary_travel_trends.pdf", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A27" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="B27" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C27" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" t="s">
-        <v>22</v>
+        <v>45</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
       </c>
       <c r="E27" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://afdc.energy.gov/files/u/publication/financial_analysis_be_transit_buses.pdf", target=_blank"&gt;Financial Analysis of Battery Electric Transit Buses. National Renewable Energy Laboratory Technical Report NREL/TP-5400-74832.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="0", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C28" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A30" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" t="s">
+        <v>101</v>
+      </c>
+      <c r="C30" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A31" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A32" t="s">
+        <v>93</v>
+      </c>
+      <c r="B32" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32" t="s">
+        <v>41</v>
+      </c>
+      <c r="D32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A33" t="s">
         <v>108</v>
       </c>
-      <c r="C28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D28" t="s">
-        <v>23</v>
-      </c>
-      <c r="E28" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.nrel.gov/docs/fy21osti/71796.pdf", target=_blank"&gt;Spatial and Temporal Analysis of the Total Cost of Ownership for Class 8 Tractors and Class 4 Parcel Delivery Trucks. National Renewable Energy Laboratory Technical Report NREL/TP-5400-71796.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>133</v>
-      </c>
-      <c r="B29" t="s">
-        <v>132</v>
-      </c>
-      <c r="C29" t="s">
-        <v>41</v>
-      </c>
-      <c r="D29" t="s">
-        <v>24</v>
-      </c>
-      <c r="E29" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.transit.dot.gov/ntd", target=_blank"&gt;National Transit Database&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="B33" t="s">
         <v>109</v>
       </c>
-      <c r="B30" t="s">
-        <v>110</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="C33" t="s">
         <v>40</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D33" t="s">
         <v>25</v>
       </c>
-      <c r="E30" t="str">
+      <c r="E33" t="str">
         <f t="shared" si="0"/>
         <v>&lt;a href="https://tedb.ornl.gov/data/", target=_blank"&gt;Transportation Energy Data Book, Edition 40.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>111</v>
-      </c>
-      <c r="B31" t="s">
-        <v>112</v>
-      </c>
-      <c r="C31" t="s">
-        <v>51</v>
-      </c>
-      <c r="D31" t="s">
-        <v>26</v>
-      </c>
-      <c r="E31" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 9: Transit Scheduling and Frequency. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>113</v>
-      </c>
-      <c r="B32" t="s">
-        <v>114</v>
-      </c>
-      <c r="C32" t="s">
-        <v>52</v>
-      </c>
-      <c r="D32" t="s">
-        <v>26</v>
-      </c>
-      <c r="E32" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 5: Vanpools and Buspools. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>115</v>
-      </c>
-      <c r="B33" t="s">
-        <v>116</v>
-      </c>
-      <c r="C33" t="s">
-        <v>53</v>
-      </c>
-      <c r="D33">
-        <v>0</v>
-      </c>
-      <c r="E33" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="0", target=_blank"&gt;Design Manual for Roads and Bridges, Volume 12, Section 2, Part 2: Induced Traffic Appraisal.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A34" t="s">
-        <v>117</v>
+        <v>61</v>
       </c>
       <c r="B34" t="s">
         <v>118</v>
       </c>
       <c r="C34" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D34" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E34" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A35" t="s">
         <v>61</v>
       </c>
@@ -2058,76 +2059,76 @@
         <v>119</v>
       </c>
       <c r="C35" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D35" t="s">
         <v>28</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A36" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B36" t="s">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="C36" t="s">
         <v>47</v>
       </c>
       <c r="D36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A37" t="s">
         <v>62</v>
       </c>
       <c r="B37" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C37" t="s">
         <v>47</v>
       </c>
       <c r="D37" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A38" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="B38" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="C38" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D38" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E38" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+        <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A39" t="s">
+        <v>120</v>
+      </c>
+      <c r="B39" t="s">
         <v>121</v>
-      </c>
-      <c r="B39" t="s">
-        <v>122</v>
       </c>
       <c r="C39" t="s">
         <v>54</v>
@@ -2140,12 +2141,12 @@
         <v>&lt;a href="https://www.itskrs.its.dot.gov/its/benecost.nsf/ID/5551ecb16b1bc9698525725f007a75d0", target=_blank"&gt;The cost of retiming traffic signals in the Washington, DC area is about $3,500 per intersection. ITS Deployment Evaluation, Intelligent Transportation Systems Joint Program Office.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A40" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C40" t="s">
         <v>55</v>
@@ -2158,12 +2159,12 @@
         <v>&lt;a href="http://www.reconnectingamerica.org/assets/Uploads/DOTClimateChangeReport-April2010-Volume1and2.pdf", target=_blank"&gt;Transportation's Role in Reducing U.S. Greenhouse Gas Emissions.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A41" t="s">
+        <v>123</v>
+      </c>
+      <c r="B41" t="s">
         <v>124</v>
-      </c>
-      <c r="B41" t="s">
-        <v>125</v>
       </c>
       <c r="C41" t="s">
         <v>47</v>
@@ -2176,12 +2177,12 @@
         <v>&lt;a href="https://www.epa.gov/climateleadership/ghg-emission-factors-hub", target=_blank"&gt;GHG Emission Factors Hub.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A42" t="s">
+        <v>125</v>
+      </c>
+      <c r="B42" t="s">
         <v>126</v>
-      </c>
-      <c r="B42" t="s">
-        <v>127</v>
       </c>
       <c r="C42" t="s">
         <v>40</v>
@@ -2194,12 +2195,12 @@
         <v>&lt;a href="https://escholarship.org/uc/item/1hh9b9mf", target=_blank"&gt;Updating the Induced Travel Calculator. National Center for Sustainable Transportation and UC Davis.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A43" t="s">
+        <v>127</v>
+      </c>
+      <c r="B43" t="s">
         <v>128</v>
-      </c>
-      <c r="B43" t="s">
-        <v>129</v>
       </c>
       <c r="C43" t="s">
         <v>45</v>
@@ -2213,6 +2214,11 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E43">
+    <sortCondition ref="A2:A43"/>
+    <sortCondition ref="B2:B43"/>
+    <sortCondition ref="C2:C43"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changes to user inputs sheet, sources xlsx, and text
</commit_message>
<xml_diff>
--- a/data/sources.xlsx
+++ b/data/sources.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aheller\Documents\GitHub\TEACART\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5305AE1-94FD-42C4-BC45-86AEDBD4C8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C33B153-BC4F-4D95-AB33-C677C9519110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{8280C5B7-8E95-43D7-B172-FB4701BB1BAF}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{8280C5B7-8E95-43D7-B172-FB4701BB1BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$42</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="134">
   <si>
     <t>https://gasprices.aaa.com/</t>
   </si>
@@ -820,14 +820,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7DB5B7-6594-4B32-9D01-0D9F2F3DF6A4}">
-  <dimension ref="A1:C43"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:C42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="57" customWidth="1"/>
-    <col min="2" max="2" width="127.6796875" customWidth="1"/>
+    <col min="2" max="2" width="127.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -838,7 +838,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="str">
         <f>Sheet2!A2</f>
         <v>[U.K.] Highways Agency</v>
@@ -852,7 +852,7 @@
         <v>1997</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="str">
         <f>Sheet2!A3</f>
         <v>American Automobile Association (AAA)</v>
@@ -866,7 +866,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="str">
         <f>Sheet2!A4</f>
         <v>American Public Transportation Association</v>
@@ -880,7 +880,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <f>Sheet2!A5</f>
         <v>Amtrak</v>
@@ -894,7 +894,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <f>Sheet2!A6</f>
         <v>Argonne National Laboratory. GREET</v>
@@ -908,7 +908,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <f>Sheet2!A7</f>
         <v>Barr, L.C.</v>
@@ -922,7 +922,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f>Sheet2!A8</f>
         <v>California Air Pollution Control Officers Association</v>
@@ -936,7 +936,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f>Sheet2!A9</f>
         <v>California Air Resources Board</v>
@@ -950,7 +950,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <f>Sheet2!A10</f>
         <v>Cambridge Systematics</v>
@@ -964,7 +964,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <f>Sheet2!A11</f>
         <v>Cesme, B., R. Roisman, and D. Miller</v>
@@ -978,7 +978,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f>Sheet2!A12</f>
         <v>Coastal Region MPO</v>
@@ -992,7 +992,7 @@
         <v>2014</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f>Sheet2!A13</f>
         <v>Evans, J.E., and R. H. Pratt, et al</v>
@@ -1006,7 +1006,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f>Sheet2!A14</f>
         <v>Evans, J.E., et al</v>
@@ -1020,7 +1020,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="str">
         <f>Sheet2!A15</f>
         <v>Federal Highway Administration</v>
@@ -1034,7 +1034,7 @@
         <v>2014</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f>Sheet2!A16</f>
         <v>Federal Highway Administration</v>
@@ -1048,7 +1048,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
         <f>Sheet2!A17</f>
         <v>Federal Highway Administration</v>
@@ -1062,7 +1062,7 @@
         <v>2013</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f>Sheet2!A18</f>
         <v>Federal Transit Administration</v>
@@ -1076,7 +1076,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f>Sheet2!A19</f>
         <v>FHWA</v>
@@ -1090,7 +1090,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f>Sheet2!A20</f>
         <v>Florida Department of Transportation</v>
@@ -1104,7 +1104,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
         <f>Sheet2!A21</f>
         <v>Hunter, C., et al</v>
@@ -1118,7 +1118,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f>Sheet2!A22</f>
         <v>Isenstadt, A., et al</v>
@@ -1132,7 +1132,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="str">
         <f>Sheet2!A23</f>
         <v>Johnson, C.; E. Nobler, L. Eudy, and M. Jeffers</v>
@@ -1146,7 +1146,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="str">
         <f>Sheet2!A24</f>
         <v>MacArthur, J., C. Cherry, M. Harpool and D. Scheppke.</v>
@@ -1160,7 +1160,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="str">
         <f>Sheet2!A25</f>
         <v>Mai, T., et al</v>
@@ -1174,7 +1174,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="str">
         <f>Sheet2!A26</f>
         <v>McGuckin, N. and A. Fucci</v>
@@ -1188,259 +1188,245 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="str">
         <f>Sheet2!A27</f>
-        <v>McGuckin, N. and A. Fucci</v>
+        <v>Mulholland, E.</v>
       </c>
       <c r="B27" t="str">
         <f>Sheet2!E27</f>
-        <v>&lt;a href="0", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
+        <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
       </c>
       <c r="C27" t="str">
         <f>Sheet2!C27</f>
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="str">
         <f>Sheet2!A28</f>
-        <v>Mulholland, E.</v>
+        <v>National Highway Traffic Safety Administration</v>
       </c>
       <c r="B28" t="str">
         <f>Sheet2!E28</f>
-        <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
+        <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
       </c>
       <c r="C28" t="str">
         <f>Sheet2!C28</f>
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="str">
         <f>Sheet2!A29</f>
-        <v>National Highway Traffic Safety Administration</v>
+        <v>New York City Clean School Bus Coalition</v>
       </c>
       <c r="B29" t="str">
         <f>Sheet2!E29</f>
-        <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
       </c>
       <c r="C29" t="str">
         <f>Sheet2!C29</f>
-        <v>2015</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.75">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="str">
         <f>Sheet2!A30</f>
-        <v>New York City Clean School Bus Coalition</v>
+        <v>NHTS</v>
       </c>
       <c r="B30" t="str">
         <f>Sheet2!E30</f>
-        <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
+        <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
       </c>
       <c r="C30" t="str">
         <f>Sheet2!C30</f>
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2009</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="str">
         <f>Sheet2!A31</f>
-        <v>NHTS</v>
+        <v>Nicholas, M.</v>
       </c>
       <c r="B31" t="str">
         <f>Sheet2!E31</f>
-        <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
+        <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
       </c>
       <c r="C31" t="str">
         <f>Sheet2!C31</f>
-        <v>2009</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="str">
         <f>Sheet2!A32</f>
-        <v>Nicholas, M.</v>
+        <v>Oak Ridge National Laboratory</v>
       </c>
       <c r="B32" t="str">
         <f>Sheet2!E32</f>
-        <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
+        <v>&lt;a href="https://tedb.ornl.gov/data/", target=_blank"&gt;Transportation Energy Data Book, Edition 40.&lt;/a&gt;</v>
       </c>
       <c r="C32" t="str">
         <f>Sheet2!C32</f>
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="str">
         <f>Sheet2!A33</f>
-        <v>Oak Ridge National Laboratory</v>
+        <v>U.S. Department of Energy</v>
       </c>
       <c r="B33" t="str">
         <f>Sheet2!E33</f>
-        <v>&lt;a href="https://tedb.ornl.gov/data/", target=_blank"&gt;Transportation Energy Data Book, Edition 40.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
       </c>
       <c r="C33" t="str">
         <f>Sheet2!C33</f>
         <v>2022</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="str">
         <f>Sheet2!A34</f>
         <v>U.S. Department of Energy</v>
       </c>
       <c r="B34" t="str">
         <f>Sheet2!E34</f>
-        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
       </c>
       <c r="C34" t="str">
         <f>Sheet2!C34</f>
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="str">
         <f>Sheet2!A35</f>
-        <v>U.S. Department of Energy</v>
+        <v>U.S. Department of Energy, Alternative Fuels Data Center</v>
       </c>
       <c r="B35" t="str">
         <f>Sheet2!E35</f>
-        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
+        <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
       </c>
       <c r="C35" t="str">
         <f>Sheet2!C35</f>
         <v>2023</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="str">
         <f>Sheet2!A36</f>
         <v>U.S. Department of Energy, Alternative Fuels Data Center</v>
       </c>
       <c r="B36" t="str">
         <f>Sheet2!E36</f>
-        <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
+        <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
       </c>
       <c r="C36" t="str">
         <f>Sheet2!C36</f>
         <v>2023</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="str">
         <f>Sheet2!A37</f>
-        <v>U.S. Department of Energy, Alternative Fuels Data Center</v>
+        <v>U.S. Department of Energy, Energy Information Administration</v>
       </c>
       <c r="B37" t="str">
         <f>Sheet2!E37</f>
-        <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
       </c>
       <c r="C37" t="str">
         <f>Sheet2!C37</f>
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="str">
         <f>Sheet2!A38</f>
-        <v>U.S. Department of Energy, Energy Information Administration</v>
+        <v>U.S. Department of Transportation</v>
       </c>
       <c r="B38" t="str">
         <f>Sheet2!E38</f>
-        <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.itskrs.its.dot.gov/its/benecost.nsf/ID/5551ecb16b1bc9698525725f007a75d0", target=_blank"&gt;The cost of retiming traffic signals in the Washington, DC area is about $3,500 per intersection. ITS Deployment Evaluation, Intelligent Transportation Systems Joint Program Office.&lt;/a&gt;</v>
       </c>
       <c r="C38" t="str">
         <f>Sheet2!C38</f>
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="str">
         <f>Sheet2!A39</f>
         <v>U.S. Department of Transportation</v>
       </c>
       <c r="B39" t="str">
         <f>Sheet2!E39</f>
-        <v>&lt;a href="https://www.itskrs.its.dot.gov/its/benecost.nsf/ID/5551ecb16b1bc9698525725f007a75d0", target=_blank"&gt;The cost of retiming traffic signals in the Washington, DC area is about $3,500 per intersection. ITS Deployment Evaluation, Intelligent Transportation Systems Joint Program Office.&lt;/a&gt;</v>
+        <v>&lt;a href="http://www.reconnectingamerica.org/assets/Uploads/DOTClimateChangeReport-April2010-Volume1and2.pdf", target=_blank"&gt;Transportation's Role in Reducing U.S. Greenhouse Gas Emissions.&lt;/a&gt;</v>
       </c>
       <c r="C39" t="str">
         <f>Sheet2!C39</f>
-        <v>2007</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="str">
         <f>Sheet2!A40</f>
-        <v>U.S. Department of Transportation</v>
+        <v>U.S. Environmental Protection Agency</v>
       </c>
       <c r="B40" t="str">
         <f>Sheet2!E40</f>
-        <v>&lt;a href="http://www.reconnectingamerica.org/assets/Uploads/DOTClimateChangeReport-April2010-Volume1and2.pdf", target=_blank"&gt;Transportation's Role in Reducing U.S. Greenhouse Gas Emissions.&lt;/a&gt;</v>
+        <v>&lt;a href="https://www.epa.gov/climateleadership/ghg-emission-factors-hub", target=_blank"&gt;GHG Emission Factors Hub.&lt;/a&gt;</v>
       </c>
       <c r="C40" t="str">
         <f>Sheet2!C40</f>
-        <v>2010</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="str">
         <f>Sheet2!A41</f>
-        <v>U.S. Environmental Protection Agency</v>
+        <v>Volker, J.N.B., and S.L. Handy</v>
       </c>
       <c r="B41" t="str">
         <f>Sheet2!E41</f>
-        <v>&lt;a href="https://www.epa.gov/climateleadership/ghg-emission-factors-hub", target=_blank"&gt;GHG Emission Factors Hub.&lt;/a&gt;</v>
+        <v>&lt;a href="https://escholarship.org/uc/item/1hh9b9mf", target=_blank"&gt;Updating the Induced Travel Calculator. National Center for Sustainable Transportation and UC Davis.&lt;/a&gt;</v>
       </c>
       <c r="C41" t="str">
         <f>Sheet2!C41</f>
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.75">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="str">
         <f>Sheet2!A42</f>
-        <v>Volker, J.N.B., and S.L. Handy</v>
+        <v>Weldon Cooper Center for Public Service, Demographics Research Group</v>
       </c>
       <c r="B42" t="str">
         <f>Sheet2!E42</f>
-        <v>&lt;a href="https://escholarship.org/uc/item/1hh9b9mf", target=_blank"&gt;Updating the Induced Travel Calculator. National Center for Sustainable Transportation and UC Davis.&lt;/a&gt;</v>
+        <v>&lt;a href="https://demographics.coopercenter.org/population-data-all-overview", target=_blank"&gt;National Population Projections.&lt;/a&gt;</v>
       </c>
       <c r="C42" t="str">
         <f>Sheet2!C42</f>
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A43" t="str">
-        <f>Sheet2!A43</f>
-        <v>Weldon Cooper Center for Public Service, Demographics Research Group</v>
-      </c>
-      <c r="B43" t="str">
-        <f>Sheet2!E43</f>
-        <v>&lt;a href="https://demographics.coopercenter.org/population-data-all-overview", target=_blank"&gt;National Population Projections.&lt;/a&gt;</v>
-      </c>
-      <c r="C43" t="str">
-        <f>Sheet2!C43</f>
         <v>2018</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C43" xr:uid="{BD7DB5B7-6594-4B32-9D01-0D9F2F3DF6A4}"/>
+  <autoFilter ref="A1:C42" xr:uid="{BD7DB5B7-6594-4B32-9D01-0D9F2F3DF6A4}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A575D46-68C3-4992-B64B-B7045A123F2A}">
-  <dimension ref="A1:E43"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:E42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="39.08984375" customWidth="1"/>
+    <col min="1" max="5" width="39.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -1457,7 +1443,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>114</v>
       </c>
@@ -1475,7 +1461,7 @@
         <v>&lt;a href="0", target=_blank"&gt;Design Manual for Roads and Bridges, Volume 12, Section 2, Part 2: Induced Traffic Appraisal.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>130</v>
       </c>
@@ -1489,11 +1475,11 @@
         <v>0</v>
       </c>
       <c r="E3" t="str">
-        <f t="shared" ref="E3:E43" si="0">_xlfn.CONCAT("&lt;a href=",CHAR(34),D3,CHAR(34),", target=_blank",CHAR(34),"&gt;",B3,"&lt;/a&gt;")</f>
+        <f t="shared" ref="E3:E42" si="0">_xlfn.CONCAT("&lt;a href=",CHAR(34),D3,CHAR(34),", target=_blank",CHAR(34),"&gt;",B3,"&lt;/a&gt;")</f>
         <v>&lt;a href="https://gasprices.aaa.com/", target=_blank"&gt;National Average Gas Prices.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -1511,7 +1497,7 @@
         <v>&lt;a href="https://www.apta.com/research-technical-resources/transit-statistics/vehicle-database/", target=_blank"&gt;Public Transportation Vehicle Database 2019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>67</v>
       </c>
@@ -1529,7 +1515,7 @@
         <v>&lt;a href="0", target=_blank"&gt;FY2019 Monthly Performance Report.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>71</v>
       </c>
@@ -1547,7 +1533,7 @@
         <v>&lt;a href="https://greet.es.anl.gov/", target=_blank"&gt;GREET (Greenhouse gases, Regulated Emissions, and Energy use in Technologies Model). Accessed 2021.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>73</v>
       </c>
@@ -1565,7 +1551,7 @@
         <v>&lt;a href="https://journals.sagepub.com/doi/10.3141/1706-01", target=_blank"&gt;Testing for the significance of induced highway travel demand in metropolitan areas. Transportation Research Record: Journal of the Transportation Research Board, vol. 1706.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>75</v>
       </c>
@@ -1583,7 +1569,7 @@
         <v>&lt;a href="https://www.airquality.org/ClimateChange/Documents/Handbook%20Public%20Draft_2021-Aug.pdf", target=_blank"&gt;Handbook for Analyzing Greenhouse Gas Emission Reductions, Assessing Climate Vulnerabilities, and Advancing Health and Equity.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -1601,7 +1587,7 @@
         <v>&lt;a href="https://ww2.arb.ca.gov/sites/default/files/classic/fuels/lcfs/guidance/lcfsguidance_20-04.pdf", target=_blank"&gt;Low Carbon Fuel Standard (LCFS) Guidance 20-04 Requesting EER-Adjusted Carbon Intensity Using a Tier 2 Pathway Application.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>83</v>
       </c>
@@ -1619,7 +1605,7 @@
         <v>&lt;a href="https://www.georgetownclimate.org/files/report/GCC_Investment_Tool.pdf", target=_blank"&gt;Transportation Investment Strategy Tool Documentation, 2023. Prepared for Georgetown Climate Center.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -1637,7 +1623,7 @@
         <v>&lt;a href="https://journals.sagepub.com/doi/10.1177/0361198118791914", target=_blank"&gt;Strategies and Barriers in Effective Bus Lane Implementation and Management: Best Practices for Use in the Greater Washington, D.C. Region. Transportation Research Record 2672:8.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>81</v>
       </c>
@@ -1655,7 +1641,7 @@
         <v>&lt;a href="https://www.thempc.org/docs/lit/corempo/studies/parkride/2014/aug/tm5.pdf", target=_blank"&gt;Park and Ride Lot Study - Technical Memorandum #5: Financial Analysis and Management Options. Prepared by Connetics Transportation Group, Moffatt &amp; Nichol, and Symbioscity.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>112</v>
       </c>
@@ -1673,7 +1659,7 @@
         <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 5: Vanpools and Buspools. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>110</v>
       </c>
@@ -1691,7 +1677,7 @@
         <v>&lt;a href="https://www.trb.org/Publications/TCRPReport95.aspx", target=_blank"&gt;TCRP Report 95, Traveler Response to Transportation System Changes. Chapter 9: Transit Scheduling and Frequency. Transportation Research Board, Washington, D.C.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>86</v>
       </c>
@@ -1709,7 +1695,7 @@
         <v>&lt;a href="http://www.pedbikesafe.org/BIKESAFE/index.cfm", target=_blank"&gt;BIKESAFE: Bicycle Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1727,7 +1713,7 @@
         <v>&lt;a href="https://www.fhwa.dot.gov/policyinformation/statistics.cfm", target=_blank"&gt;Highway Statistics Series, 2019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>86</v>
       </c>
@@ -1745,7 +1731,7 @@
         <v>&lt;a href="http://www.pedbikesafe.org/PEDSAFE/index.cfm", target=_blank"&gt;PEDSAFE: Pedestrian Safety Guide and Countermeasure Selection System.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>132</v>
       </c>
@@ -1763,7 +1749,7 @@
         <v>&lt;a href="https://www.transit.dot.gov/ntd", target=_blank"&gt;National Transit Database&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>60</v>
       </c>
@@ -1781,7 +1767,7 @@
         <v>&lt;a href="https://faf.ornl.gov/faf5/", target=_blank"&gt;Freight Analysis Framework Version 5.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>84</v>
       </c>
@@ -1799,7 +1785,7 @@
         <v>&lt;a href="https://www.fdot.gov/programmanagement/estimates/documents/costpermilemodelsreports", target=_blank"&gt;Cost Per Mile Models Reports. Accessed June 2023.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>106</v>
       </c>
@@ -1817,7 +1803,7 @@
         <v>&lt;a href="https://www.nrel.gov/docs/fy21osti/71796.pdf", target=_blank"&gt;Spatial and Temporal Analysis of the Total Cost of Ownership for Class 8 Tractors and Class 4 Parcel Delivery Trucks. National Renewable Energy Laboratory Technical Report NREL/TP-5400-71796.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -1835,7 +1821,7 @@
         <v>&lt;a href="https://theicct.org/publication/real-world-phev-us-dec22/", target=_blank"&gt;Real World Usage of Plug-In Hybrid Electric Vehicles. International Council on Clean Transportation.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>104</v>
       </c>
@@ -1853,7 +1839,7 @@
         <v>&lt;a href="https://afdc.energy.gov/files/u/publication/financial_analysis_be_transit_buses.pdf", target=_blank"&gt;Financial Analysis of Battery Electric Transit Buses. National Renewable Energy Laboratory Technical Report NREL/TP-5400-74832.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>99</v>
       </c>
@@ -1871,7 +1857,7 @@
         <v>&lt;a href="https://pdxscholar.library.pdx.edu/trec_reports/161/", target=_blank"&gt;A North American Survey of Electric Bicycle Owners. NITC-RR-1041. Portland, OR: Transportation Research and Education Center (TREC). https://dx.doi.org/10.15760/ trec.197&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>102</v>
       </c>
@@ -1889,7 +1875,7 @@
         <v>&lt;a href="https://www.nrel.gov/docs/fy18osti/71500.pdf", target=_blank"&gt;Electrification Futures Study: Scenarios of Electric Technology Adoption and Power Consumption for the United States. Golden, CO: National Renewable Energy Laboratory. NREL/TP-6A20-71500.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>89</v>
       </c>
@@ -1907,317 +1893,299 @@
         <v>&lt;a href="https://nhts.ornl.gov/assets/2017_nhts_summary_travel_trends.pdf", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27">
+        <v>40</v>
+      </c>
+      <c r="D27" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28">
         <v>0</v>
       </c>
-      <c r="E27" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="0", target=_blank"&gt;Summary of Travel Trends: 2017 National Household Travel Survey. U.S. Department of Transportation, Federal Highway Administration, FHWA-PL-18-019.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.75">
-      <c r="A28" t="s">
-        <v>97</v>
-      </c>
-      <c r="B28" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="E28" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" t="s">
+        <v>101</v>
+      </c>
+      <c r="C29" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" t="s">
+        <v>49</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" t="s">
+        <v>41</v>
+      </c>
+      <c r="D31" t="s">
+        <v>15</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C32" t="s">
         <v>40</v>
       </c>
-      <c r="D28" t="s">
-        <v>17</v>
-      </c>
-      <c r="E28" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://theicct.org/wp-content/uploads/2022/01/cost-ev-vans-pickups-us-2040-jan22.pdf", target=_blank"&gt;Cost of electric commercial vans and pickup trucks in the United States through 2040. International Council on Clean Transportation Working Paper 2022-01.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.75">
-      <c r="A29" t="s">
-        <v>57</v>
-      </c>
-      <c r="B29" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29" t="s">
-        <v>50</v>
-      </c>
-      <c r="D29">
-        <v>0</v>
-      </c>
-      <c r="E29" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="0", target=_blank"&gt;National Traffic Speeds Survey&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.75">
-      <c r="A30" t="s">
-        <v>19</v>
-      </c>
-      <c r="B30" t="s">
-        <v>101</v>
-      </c>
-      <c r="C30" t="s">
-        <v>65</v>
-      </c>
-      <c r="D30" t="s">
-        <v>20</v>
-      </c>
-      <c r="E30" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.nycschoolbus.org/technical-school-bus-need-to-know-1#:~:text=The%20cost%20of%20an%20electric,in%20between%20%2490%2C000%20to%20%24110%2C000.", target=_blank"&gt;3 Types of Electric School Buses.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.75">
-      <c r="A31" t="s">
-        <v>56</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C31" t="s">
-        <v>49</v>
-      </c>
-      <c r="D31">
-        <v>0</v>
-      </c>
-      <c r="E31" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;a href="0", target=_blank"&gt;National Household Travel Survey&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.75">
-      <c r="A32" t="s">
-        <v>93</v>
-      </c>
-      <c r="B32" t="s">
-        <v>94</v>
-      </c>
-      <c r="C32" t="s">
-        <v>41</v>
-      </c>
       <c r="D32" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E32" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://theicct.org/sites/default/files/publications/ICCT_EV_Charging_Cost_20190813.pdf", target=_blank"&gt;Estimating electric vehicle charging infrastructure costs across major U.S. metropolitan areas. International Council on Clean Transportation Working Paper 2019-14.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://tedb.ornl.gov/data/", target=_blank"&gt;Transportation Energy Data Book, Edition 40.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>108</v>
+        <v>61</v>
       </c>
       <c r="B33" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="C33" t="s">
         <v>40</v>
       </c>
       <c r="D33" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E33" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://tedb.ornl.gov/data/", target=_blank"&gt;Transportation Energy Data Book, Edition 40.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>61</v>
       </c>
       <c r="B34" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C34" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D34" t="s">
         <v>28</v>
       </c>
       <c r="E34" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2022. Energy Information Administration.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B35" t="s">
-        <v>119</v>
+        <v>63</v>
       </c>
       <c r="C35" t="s">
         <v>47</v>
       </c>
       <c r="D35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.eia.gov/outlooks/aeo/", target=_blank"&gt;Annual Energy Outlook Reference Case 2023. Energy Information Administration.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>62</v>
       </c>
       <c r="B36" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C36" t="s">
         <v>47</v>
       </c>
       <c r="D36" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://afdc.energy.gov/data", target=_blank"&gt;Average Fuel Economy by Major Vehicle Category&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="B37" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="C37" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D37" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://afdc.energy.gov/tools", target=_blank"&gt;Fuel Properties Comparison&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B38" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C38" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D38" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E38" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.eia.gov/electricity/state/", target=_blank"&gt;US Electricity Profile 2021.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://www.itskrs.its.dot.gov/its/benecost.nsf/ID/5551ecb16b1bc9698525725f007a75d0", target=_blank"&gt;The cost of retiming traffic signals in the Washington, DC area is about $3,500 per intersection. ITS Deployment Evaluation, Intelligent Transportation Systems Joint Program Office.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>120</v>
       </c>
       <c r="B39" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C39" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D39" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E39" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.itskrs.its.dot.gov/its/benecost.nsf/ID/5551ecb16b1bc9698525725f007a75d0", target=_blank"&gt;The cost of retiming traffic signals in the Washington, DC area is about $3,500 per intersection. ITS Deployment Evaluation, Intelligent Transportation Systems Joint Program Office.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="http://www.reconnectingamerica.org/assets/Uploads/DOTClimateChangeReport-April2010-Volume1and2.pdf", target=_blank"&gt;Transportation's Role in Reducing U.S. Greenhouse Gas Emissions.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B40" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C40" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D40" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E40" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="http://www.reconnectingamerica.org/assets/Uploads/DOTClimateChangeReport-April2010-Volume1and2.pdf", target=_blank"&gt;Transportation's Role in Reducing U.S. Greenhouse Gas Emissions.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://www.epa.gov/climateleadership/ghg-emission-factors-hub", target=_blank"&gt;GHG Emission Factors Hub.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B41" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C41" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="D41" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E41" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://www.epa.gov/climateleadership/ghg-emission-factors-hub", target=_blank"&gt;GHG Emission Factors Hub.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.75">
+        <v>&lt;a href="https://escholarship.org/uc/item/1hh9b9mf", target=_blank"&gt;Updating the Induced Travel Calculator. National Center for Sustainable Transportation and UC Davis.&lt;/a&gt;</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B42" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C42" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D42" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E42" t="str">
         <f t="shared" si="0"/>
-        <v>&lt;a href="https://escholarship.org/uc/item/1hh9b9mf", target=_blank"&gt;Updating the Induced Travel Calculator. National Center for Sustainable Transportation and UC Davis.&lt;/a&gt;</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.75">
-      <c r="A43" t="s">
-        <v>127</v>
-      </c>
-      <c r="B43" t="s">
-        <v>128</v>
-      </c>
-      <c r="C43" t="s">
-        <v>45</v>
-      </c>
-      <c r="D43" t="s">
-        <v>35</v>
-      </c>
-      <c r="E43" t="str">
-        <f t="shared" si="0"/>
         <v>&lt;a href="https://demographics.coopercenter.org/population-data-all-overview", target=_blank"&gt;National Population Projections.&lt;/a&gt;</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E43">
-    <sortCondition ref="A2:A43"/>
-    <sortCondition ref="B2:B43"/>
-    <sortCondition ref="C2:C43"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E42">
+    <sortCondition ref="A2:A42"/>
+    <sortCondition ref="B2:B42"/>
+    <sortCondition ref="C2:C42"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>